<commit_message>
tambahkan fitur upload gambar di halaman edit tamu
</commit_message>
<xml_diff>
--- a/Laporan Buku Tamu.xlsx
+++ b/Laporan Buku Tamu.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
   <si>
     <t>No</t>
   </si>
@@ -72,6 +72,21 @@
   </si>
   <si>
     <t>Kerkom</t>
+  </si>
+  <si>
+    <t>Udin</t>
+  </si>
+  <si>
+    <t>Bojong</t>
+  </si>
+  <si>
+    <t>089920091341</t>
+  </si>
+  <si>
+    <t>Zeus</t>
+  </si>
+  <si>
+    <t>Final Boss</t>
   </si>
 </sst>
 </file>
@@ -411,7 +426,7 @@
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:G4"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" spans="1:7">
@@ -481,6 +496,29 @@
       </c>
       <c r="G3" t="s">
         <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+      <c r="F4" t="s">
+        <v>22</v>
+      </c>
+      <c r="G4" t="s">
+        <v>23</v>
       </c>
     </row>
   </sheetData>

</xml_diff>